<commit_message>
Bỏ dòng chú thích (*) không còn dùng trong bảng Excel
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JLkhnZKuapW5Zj7yjV8vMu
</commit_message>
<xml_diff>
--- a/Du an PTN cao hoc Hoa hoc/Bang 1 - danh muc thiet bi va gia.xlsx
+++ b/Du an PTN cao hoc Hoa hoc/Bang 1 - danh muc thiet bi va gia.xlsx
@@ -1085,12 +1085,7 @@
       <c r="E31" s="8" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" t="inlineStr"/>
-      <c r="B32" s="9" t="inlineStr">
-        <is>
-          <t>(*) Đơn giá ước lượng, chưa có báo giá.</t>
-        </is>
-      </c>
+      <c r="B32" s="9" t="n"/>
       <c r="D32" s="8" t="n"/>
       <c r="E32" s="8" t="n"/>
     </row>

</xml_diff>

<commit_message>
Áp phương án cắt giảm: tổng Bảng 1 còn 14.644.310.000 đồng
Bỏ máy đo kích thước hạt/thế zeta và hệ đo độ hòa tan; TGA-FTIR thay bằng TGA; đông khô, UV-Vis, lò ống còn 01; bổ sung lò nung buồng, tủ hóa chất, máy đo pH, khuấy cơ, máy phân tích độ ẩm, bể điều nhiệt. Cập nhật Bảng 2, mục I.5, I.6, V.1, VII và bảng Excel.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JLkhnZKuapW5Zj7yjV8vMu
</commit_message>
<xml_diff>
--- a/Du an PTN cao hoc Hoa hoc/Bang 1 - danh muc thiet bi va gia.xlsx
+++ b/Du an PTN cao hoc Hoa hoc/Bang 1 - danh muc thiet bi va gia.xlsx
@@ -469,7 +469,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E32"/>
+  <dimension ref="A1:E34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -776,7 +776,7 @@
         </is>
       </c>
       <c r="C15" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D15" s="4" t="n">
         <v>900000000</v>
@@ -856,7 +856,7 @@
         </is>
       </c>
       <c r="C19" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D19" s="4" t="n">
         <v>500000000</v>
@@ -872,14 +872,14 @@
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>Máy quang phổ UV-Vis hai chùm tia</t>
+          <t>Lò nung buồng 1.100 °C</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D20" s="4" t="n">
-        <v>200000000</v>
+        <v>323090000</v>
       </c>
       <c r="E20" s="4">
         <f>C20*D20</f>
@@ -892,14 +892,14 @@
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>Máy sắc ký khí (FID, TCD)</t>
+          <t>Tủ đựng hóa chất có lọc than hoạt tính</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D21" s="4" t="n">
-        <v>2200000000</v>
+        <v>90000000</v>
       </c>
       <c r="E21" s="4">
         <f>C21*D21</f>
@@ -912,14 +912,14 @@
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>Máy đo kích thước hạt và thế zeta</t>
+          <t>Máy đo pH để bàn</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
         <v>1</v>
       </c>
       <c r="D22" s="4" t="n">
-        <v>4389940000</v>
+        <v>35360000</v>
       </c>
       <c r="E22" s="4">
         <f>C22*D22</f>
@@ -932,14 +932,14 @@
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>Hệ phân tích nhiệt trọng lượng ghép nối FTIR (TGA-FTIR)</t>
+          <t>Máy khuấy cơ</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D23" s="4" t="n">
-        <v>3200000000</v>
+        <v>52700000</v>
       </c>
       <c r="E23" s="4">
         <f>C23*D23</f>
@@ -952,14 +952,14 @@
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>Máy quang phổ hấp thụ nguyên tử (AAS) ngọn lửa</t>
+          <t>Máy phân tích độ ẩm</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
         <v>1</v>
       </c>
       <c r="D24" s="4" t="n">
-        <v>1500000000</v>
+        <v>27500000</v>
       </c>
       <c r="E24" s="4">
         <f>C24*D24</f>
@@ -972,14 +972,14 @@
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>Máy thử kéo vạn năng</t>
+          <t>Bể điều nhiệt 45 L</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
         <v>1</v>
       </c>
       <c r="D25" s="4" t="n">
-        <v>800000000</v>
+        <v>60040000</v>
       </c>
       <c r="E25" s="4">
         <f>C25*D25</f>
@@ -992,14 +992,14 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>Máy đo điện trở mặt 4 mũi dò</t>
+          <t>Máy quang phổ UV-Vis hai chùm tia</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
         <v>1</v>
       </c>
       <c r="D26" s="4" t="n">
-        <v>300000000</v>
+        <v>200000000</v>
       </c>
       <c r="E26" s="4">
         <f>C26*D26</f>
@@ -1012,14 +1012,14 @@
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>Máy quang phổ huỳnh quang</t>
+          <t>Máy sắc ký khí (FID, TCD)</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
         <v>1</v>
       </c>
       <c r="D27" s="4" t="n">
-        <v>1500000000</v>
+        <v>2200000000</v>
       </c>
       <c r="E27" s="4">
         <f>C27*D27</f>
@@ -1032,14 +1032,14 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>Hệ đo độ hòa tan 8 vị trí kèm lấy mẫu tự động</t>
+          <t>Máy phân tích nhiệt trọng lượng (TGA)</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
         <v>1</v>
       </c>
       <c r="D28" s="4" t="n">
-        <v>3000000000</v>
+        <v>1300000000</v>
       </c>
       <c r="E28" s="4">
         <f>C28*D28</f>
@@ -1052,14 +1052,14 @@
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>Máy đo điện hóa đa kênh (potentiostat/galvanostat)</t>
+          <t>Máy quang phổ hấp thụ nguyên tử (AAS) ngọn lửa</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
         <v>1</v>
       </c>
       <c r="D29" s="4" t="n">
-        <v>500000000</v>
+        <v>1500000000</v>
       </c>
       <c r="E29" s="4">
         <f>C29*D29</f>
@@ -1067,27 +1067,98 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="5" t="inlineStr"/>
-      <c r="B30" s="6" t="inlineStr">
+      <c r="A30" s="2" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>Máy thử kéo vạn năng</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D30" s="4" t="n">
+        <v>800000000</v>
+      </c>
+      <c r="E30" s="4">
+        <f>C30*D30</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>Máy đo điện trở mặt 4 mũi dò</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D31" s="4" t="n">
+        <v>300000000</v>
+      </c>
+      <c r="E31" s="4">
+        <f>C31*D31</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>Máy quang phổ huỳnh quang</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D32" s="4" t="n">
+        <v>1500000000</v>
+      </c>
+      <c r="E32" s="4">
+        <f>C32*D32</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>Máy đo điện hóa đa kênh (potentiostat/galvanostat)</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D33" s="4" t="n">
+        <v>500000000</v>
+      </c>
+      <c r="E33" s="4">
+        <f>C33*D33</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr"/>
+      <c r="B34" s="6" t="inlineStr">
         <is>
           <t>TỔNG CỘNG</t>
         </is>
       </c>
-      <c r="C30" s="5" t="inlineStr"/>
-      <c r="D30" s="7" t="inlineStr"/>
-      <c r="E30" s="7">
-        <f>SUM(E2:E29)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="31">
-      <c r="D31" s="8" t="n"/>
-      <c r="E31" s="8" t="n"/>
-    </row>
-    <row r="32">
-      <c r="B32" s="9" t="n"/>
-      <c r="D32" s="8" t="n"/>
-      <c r="E32" s="8" t="n"/>
+      <c r="C34" s="5" t="inlineStr"/>
+      <c r="D34" s="7" t="inlineStr"/>
+      <c r="E34" s="7">
+        <f>SUM(E2:E33)</f>
+        <v/>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>